<commit_message>
Temporary commit to apply stash safely
</commit_message>
<xml_diff>
--- a/src/test/resources/DieticianAppExcelData.xlsx
+++ b/src/test/resources/DieticianAppExcelData.xlsx
@@ -5,38 +5,28 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\saphi\eclipse-workspace\Team2BDDSeleniumHackathon\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mahaj\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A39277AA-18B8-452D-AF32-1B1AEBE24543}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39EA271F-751F-4F89-9B8D-2D53B36A33FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1695" yWindow="1530" windowWidth="21600" windowHeight="11055" xr2:uid="{76D14252-9C01-4834-806D-51F1D7703778}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{76D14252-9C01-4834-806D-51F1D7703778}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginPageContent" sheetId="1" r:id="rId1"/>
+    <sheet name="AddPatientData" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="145">
   <si>
     <t>username</t>
   </si>
@@ -114,13 +104,370 @@
   </si>
   <si>
     <t>initiates login</t>
+  </si>
+  <si>
+    <t>invalidData</t>
+  </si>
+  <si>
+    <t>first_name</t>
+  </si>
+  <si>
+    <t>last_name</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>contact</t>
+  </si>
+  <si>
+    <t>allergy</t>
+  </si>
+  <si>
+    <t>food_preference</t>
+  </si>
+  <si>
+    <t>cuisine</t>
+  </si>
+  <si>
+    <t>dob</t>
+  </si>
+  <si>
+    <t>weight</t>
+  </si>
+  <si>
+    <t>height</t>
+  </si>
+  <si>
+    <t>temperature</t>
+  </si>
+  <si>
+    <t>sp</t>
+  </si>
+  <si>
+    <t>dp</t>
+  </si>
+  <si>
+    <t>expected_Message</t>
+  </si>
+  <si>
+    <t>first name with numeric data</t>
+  </si>
+  <si>
+    <t>12345</t>
+  </si>
+  <si>
+    <t>Tank</t>
+  </si>
+  <si>
+    <t>Anthem.Tank@email.com</t>
+  </si>
+  <si>
+    <t>9876543210</t>
+  </si>
+  <si>
+    <t>Peanuts</t>
+  </si>
+  <si>
+    <t>Vegan</t>
+  </si>
+  <si>
+    <t>Punjabi</t>
+  </si>
+  <si>
+    <t>04/20/21985</t>
+  </si>
+  <si>
+    <t>75</t>
+  </si>
+  <si>
+    <t>175</t>
+  </si>
+  <si>
+    <t>98.6</t>
+  </si>
+  <si>
+    <t>120</t>
+  </si>
+  <si>
+    <t>80</t>
+  </si>
+  <si>
+    <t>Patient first name accepts only alphabets</t>
+  </si>
+  <si>
+    <t>first name with special character data</t>
+  </si>
+  <si>
+    <t>Anthem@#!</t>
+  </si>
+  <si>
+    <t>Mandatory check for firstname field</t>
+  </si>
+  <si>
+    <t>Firstname field is required</t>
+  </si>
+  <si>
+    <t>last name with  numeric data</t>
+  </si>
+  <si>
+    <t>Anthem</t>
+  </si>
+  <si>
+    <t>Patient last name accepts only alphabets</t>
+  </si>
+  <si>
+    <t>last name with special character data</t>
+  </si>
+  <si>
+    <t>%&amp;$%</t>
+  </si>
+  <si>
+    <t>Mandatory field check for lastname field</t>
+  </si>
+  <si>
+    <t>Lastname field is required</t>
+  </si>
+  <si>
+    <t>email with  starts with number</t>
+  </si>
+  <si>
+    <t>1abc@example.com</t>
+  </si>
+  <si>
+    <t>Please enter a valid email address</t>
+  </si>
+  <si>
+    <t>email without @ symbol</t>
+  </si>
+  <si>
+    <t>abcexample.com</t>
+  </si>
+  <si>
+    <t>email with special characters</t>
+  </si>
+  <si>
+    <t>abc@exa!mple.com</t>
+  </si>
+  <si>
+    <t>email without .com</t>
+  </si>
+  <si>
+    <t>abc@example</t>
+  </si>
+  <si>
+    <t>Existing email id</t>
+  </si>
+  <si>
+    <t>existing@example.com</t>
+  </si>
+  <si>
+    <t>Email id already exists</t>
+  </si>
+  <si>
+    <t>Mandatory check for email field</t>
+  </si>
+  <si>
+    <t>Email field is required</t>
+  </si>
+  <si>
+    <t>contact no. with alphabets</t>
+  </si>
+  <si>
+    <t>abcdef</t>
+  </si>
+  <si>
+    <t>Contact number accepts only numeric values</t>
+  </si>
+  <si>
+    <t>contact no. with special characters</t>
+  </si>
+  <si>
+    <t>98765@#!</t>
+  </si>
+  <si>
+    <t>contact no. with less than ten digits</t>
+  </si>
+  <si>
+    <t>123</t>
+  </si>
+  <si>
+    <t>Please enter a valid contact number</t>
+  </si>
+  <si>
+    <t>contact no. with greater than ten digits</t>
+  </si>
+  <si>
+    <t>123456789012</t>
+  </si>
+  <si>
+    <t>Existing contact number</t>
+  </si>
+  <si>
+    <t>Contact number already exists</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mandatory field check for contact num </t>
+  </si>
+  <si>
+    <t>Contact Num is required</t>
+  </si>
+  <si>
+    <t>Leaving Allergies field empty</t>
+  </si>
+  <si>
+    <t>Allergies is required</t>
+  </si>
+  <si>
+    <t>Leaving Food Preference field empty</t>
+  </si>
+  <si>
+    <t>Food Preference is required</t>
+  </si>
+  <si>
+    <t>Leaving Cusine Category field empty</t>
+  </si>
+  <si>
+    <t>76</t>
+  </si>
+  <si>
+    <t>Cuisine Category is required</t>
+  </si>
+  <si>
+    <t>Leaving DOB field empty</t>
+  </si>
+  <si>
+    <t>77</t>
+  </si>
+  <si>
+    <t>Date is required</t>
+  </si>
+  <si>
+    <t>Add weight with valid data</t>
+  </si>
+  <si>
+    <t>176</t>
+  </si>
+  <si>
+    <t>Patient successfully created</t>
+  </si>
+  <si>
+    <t>Add weight with special characters</t>
+  </si>
+  <si>
+    <t>#!@</t>
+  </si>
+  <si>
+    <t>177</t>
+  </si>
+  <si>
+    <t>Please enter a valid weight</t>
+  </si>
+  <si>
+    <t>Add weight with alphabets</t>
+  </si>
+  <si>
+    <t>seventy</t>
+  </si>
+  <si>
+    <t>98.7</t>
+  </si>
+  <si>
+    <t>Add height with valid data</t>
+  </si>
+  <si>
+    <t>98.8</t>
+  </si>
+  <si>
+    <t>Add height with special characters</t>
+  </si>
+  <si>
+    <t>#78@</t>
+  </si>
+  <si>
+    <t>121</t>
+  </si>
+  <si>
+    <t>Please enter a valid height</t>
+  </si>
+  <si>
+    <t>Add height with alphabets</t>
+  </si>
+  <si>
+    <t>tall</t>
+  </si>
+  <si>
+    <t>122</t>
+  </si>
+  <si>
+    <t>Add temperature with valid data</t>
+  </si>
+  <si>
+    <t>Add temperature with special characters</t>
+  </si>
+  <si>
+    <t>@#$</t>
+  </si>
+  <si>
+    <t>Please enter a valid temperature</t>
+  </si>
+  <si>
+    <t>Add temperature with alphabets</t>
+  </si>
+  <si>
+    <t>hot</t>
+  </si>
+  <si>
+    <t>low</t>
+  </si>
+  <si>
+    <t>Add SP,DP with special characters</t>
+  </si>
+  <si>
+    <t>Please enter a valid SP value</t>
+  </si>
+  <si>
+    <t>Add SP ,DP with alphabets</t>
+  </si>
+  <si>
+    <t>high</t>
+  </si>
+  <si>
+    <t>Add SP,DP with valid data</t>
+  </si>
+  <si>
+    <t>all fields with valid data</t>
+  </si>
+  <si>
+    <t>Atlas</t>
+  </si>
+  <si>
+    <t>Tilak</t>
+  </si>
+  <si>
+    <t>atlastilak@gzmail.com</t>
+  </si>
+  <si>
+    <t>Milk</t>
+  </si>
+  <si>
+    <t>patient created with mandatory filds only</t>
+  </si>
+  <si>
+    <t>Anny</t>
+  </si>
+  <si>
+    <t>Car</t>
+  </si>
+  <si>
+    <t>anycar@cars.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -136,16 +483,64 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF7B0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1A6B2E"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF2E3F8F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFDDEDE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD6F0DC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -153,11 +548,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -165,8 +576,36 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="6" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -500,16 +939,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9ED2C843-2039-4D8A-A327-D6CA78F0293A}">
   <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="29.53125" customWidth="1"/>
-    <col min="2" max="2" width="17.9296875" customWidth="1"/>
-    <col min="3" max="3" width="19.3984375" customWidth="1"/>
+    <col min="1" max="1" width="29.54296875" customWidth="1"/>
+    <col min="2" max="2" width="17.90625" customWidth="1"/>
+    <col min="3" max="3" width="19.36328125" customWidth="1"/>
     <col min="4" max="4" width="23" customWidth="1"/>
-    <col min="5" max="5" width="26.3984375" customWidth="1"/>
+    <col min="5" max="5" width="26.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
@@ -526,7 +965,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -543,7 +982,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>7</v>
       </c>
@@ -560,7 +999,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -577,7 +1016,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
@@ -594,7 +1033,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
@@ -611,7 +1050,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>16</v>
       </c>
@@ -626,7 +1065,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>18</v>
       </c>
@@ -641,7 +1080,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>20</v>
       </c>
@@ -662,4 +1101,1738 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C7168DD-AD97-4A85-92A6-70146638992A}">
+  <dimension ref="A1:O37"/>
+  <sheetFormatPr defaultRowHeight="41.5" customHeight="1" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="28.90625" customWidth="1"/>
+    <col min="5" max="5" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.90625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="17.08984375" style="10" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="I1" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="L1" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="M1" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="O1" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N2" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O2" s="8" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K3" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L3" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M3" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O3" s="8" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M4" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O4" s="8" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" s="5">
+        <v>123</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I5" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L5" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M5" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O5" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M6" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O6" s="8" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L7" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M7" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N7" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O7" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I8" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J8" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K8" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L8" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M8" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N8" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O8" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L9" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M9" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N9" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O9" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G10" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I10" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J10" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K10" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L10" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M10" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N10" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O10" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J11" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K11" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M11" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N11" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O11" s="8" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I12" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J12" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K12" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L12" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M12" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N12" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O12" s="8" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J13" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K13" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L13" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M13" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N13" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O13" s="8" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I14" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J14" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K14" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L14" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M14" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N14" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O14" s="8" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I15" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J15" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K15" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L15" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M15" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N15" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O15" s="8" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J16" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K16" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L16" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M16" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N16" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O16" s="8" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J17" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K17" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L17" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M17" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N17" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O17" s="8" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H18" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I18" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J18" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K18" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L18" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M18" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N18" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O18" s="8" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E19" s="5"/>
+      <c r="F19" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I19" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J19" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K19" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L19" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M19" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N19" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O19" s="8" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H20" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I20" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J20" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K20" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L20" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M20" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N20" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O20" s="8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F21" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I21" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J21" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K21" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L21" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M21" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N21" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O21" s="8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F22" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G22" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H22" s="5"/>
+      <c r="I22" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J22" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="K22" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L22" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M22" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N22" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O22" s="8" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G23" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I23" s="5"/>
+      <c r="J23" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="K23" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L23" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M23" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N23" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O23" s="8" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="E24" s="6">
+        <v>8987670000</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="I24" s="6">
+        <v>31164</v>
+      </c>
+      <c r="J24" s="6">
+        <v>70</v>
+      </c>
+      <c r="K24" s="6">
+        <v>165</v>
+      </c>
+      <c r="L24" s="6">
+        <v>98.6</v>
+      </c>
+      <c r="M24" s="6">
+        <v>120</v>
+      </c>
+      <c r="N24" s="6">
+        <v>80</v>
+      </c>
+      <c r="O24" s="9"/>
+    </row>
+    <row r="25" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="I25" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="J25" s="6">
+        <v>71</v>
+      </c>
+      <c r="K25" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="L25" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="M25" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="N25" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="O25" s="9" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G26" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I26" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J26" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="K26" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="L26" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M26" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N26" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O26" s="8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G27" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H27" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I27" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J27" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="K27" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L27" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="M27" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N27" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O27" s="8" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="I28" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="J28" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="K28" s="6">
+        <v>175</v>
+      </c>
+      <c r="L28" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="M28" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="N28" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="O28" s="9" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G29" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H29" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I29" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J29" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K29" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="L29" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M29" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="N29" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O29" s="8" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G30" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H30" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I30" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J30" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K30" s="5" t="s">
+        <v>122</v>
+      </c>
+      <c r="L30" s="5">
+        <v>98.6</v>
+      </c>
+      <c r="M30" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="N30" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="O30" s="8" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F31" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="I31" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="J31" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="K31" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="L31" s="6">
+        <v>99.6</v>
+      </c>
+      <c r="M31" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="N31" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="O31" s="9" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E32" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F32" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G32" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H32" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I32" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J32" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K32" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L32" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="M32" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N32" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="O32" s="8" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D33" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E33" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F33" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H33" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I33" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J33" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K33" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L33" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="M33" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="N33" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="O33" s="8" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F34" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G34" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H34" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I34" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J34" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K34" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L34" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M34" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="N34" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="O34" s="8" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="E35" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F35" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G35" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="H35" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="I35" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="J35" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="K35" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="L35" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="M35" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="N35" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="O35" s="8" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="G36" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="H36" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="I36" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="J36" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="K36" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="L36" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="M36" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="N36" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="O36" s="9" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15" ht="41.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="E37" s="6">
+        <v>1231231234</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="G37" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="I37" s="11">
+        <v>31080</v>
+      </c>
+      <c r="J37" s="6"/>
+      <c r="K37" s="6"/>
+      <c r="L37" s="6"/>
+      <c r="M37" s="6"/>
+      <c r="N37" s="6"/>
+      <c r="O37" s="9" t="s">
+        <v>107</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D31" r:id="rId1" display="Anthem.doe@email.com" xr:uid="{2F1E5DCB-2662-4AE4-A68C-7F7942607782}"/>
+    <hyperlink ref="J26" r:id="rId2" xr:uid="{592CC3C0-1FA1-4139-B81A-430409CAC14E}"/>
+    <hyperlink ref="K29" r:id="rId3" xr:uid="{10366812-2C4A-4FFF-9C47-1EF6CF0AE3F9}"/>
+    <hyperlink ref="D24" r:id="rId4" xr:uid="{5F8BB14F-9B3F-4D5A-92BD-213D7E2DF31E}"/>
+    <hyperlink ref="D37" r:id="rId5" xr:uid="{9512357B-AD5D-4C72-9D3B-4BC2E891FA1E}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>